<commit_message>
Added initial Turing test analysis
</commit_message>
<xml_diff>
--- a/turing_test/turing_mapping.xlsx
+++ b/turing_test/turing_mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://technionmail-my.sharepoint.com/personal/rmaya_campus_technion_ac_il/Documents/Uni/Semester 8/ML Project/audio_clips/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://technionmail-my.sharepoint.com/personal/rmaya_campus_technion_ac_il/Documents/Uni/Semester 8/ML Project/Code/disfluency-insertion/turing_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="102" documentId="11_0F590EFC617043BAC26544B40A73EC487892CCA6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22B18A71-579F-4BD6-B246-8417B15F742D}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="11_0F590EFC617043BAC26544B40A73EC487892CCA6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C90FBC8A-AFED-4B7E-9B20-B9A274F3ABEA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>P1</t>
   </si>
@@ -51,15 +51,6 @@
     <t>sample_num</t>
   </si>
   <si>
-    <t>llm_human_order</t>
-  </si>
-  <si>
-    <t>h_l</t>
-  </si>
-  <si>
-    <t>l_h</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -85,6 +76,12 @@
   </si>
   <si>
     <t>&gt;0.5</t>
+  </si>
+  <si>
+    <t>human_clip</t>
+  </si>
+  <si>
+    <t>P_id</t>
   </si>
 </sst>
 </file>
@@ -143,6 +140,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -419,20 +420,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
       <c r="B1" t="s">
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -443,16 +447,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -463,16 +467,16 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -483,7 +487,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -494,7 +498,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -505,7 +509,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -516,7 +520,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -527,7 +531,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>